<commit_message>
cositas de la nueva empresa
</commit_message>
<xml_diff>
--- a/productos_no_ml.xlsx
+++ b/productos_no_ml.xlsx
@@ -14,63 +14,45 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>sku</t>
   </si>
   <si>
-    <t>959714</t>
+    <t>044373</t>
+  </si>
+  <si>
+    <t>621761</t>
+  </si>
+  <si>
+    <t>616236</t>
+  </si>
+  <si>
+    <t>008206</t>
+  </si>
+  <si>
+    <t>368103</t>
+  </si>
+  <si>
+    <t>044495</t>
+  </si>
+  <si>
+    <t>579287</t>
+  </si>
+  <si>
+    <t>253505</t>
   </si>
   <si>
     <t>097208</t>
   </si>
   <si>
-    <t>528180</t>
-  </si>
-  <si>
-    <t>124247</t>
-  </si>
-  <si>
-    <t>201069</t>
-  </si>
-  <si>
-    <t>621761</t>
-  </si>
-  <si>
-    <t>812857</t>
-  </si>
-  <si>
-    <t>675543</t>
-  </si>
-  <si>
-    <t>274669</t>
-  </si>
-  <si>
-    <t>942668</t>
+    <t>402612</t>
+  </si>
+  <si>
+    <t>179541</t>
   </si>
   <si>
     <t>127221</t>
-  </si>
-  <si>
-    <t>876119</t>
-  </si>
-  <si>
-    <t>129780</t>
-  </si>
-  <si>
-    <t>534786</t>
-  </si>
-  <si>
-    <t>640773</t>
-  </si>
-  <si>
-    <t>164365</t>
-  </si>
-  <si>
-    <t>368103</t>
-  </si>
-  <si>
-    <t>044373</t>
   </si>
 </sst>
 </file>
@@ -428,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -496,36 +478,6 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:1">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1">
-      <c r="A17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1">
-      <c r="A19" t="s">
-        <v>18</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>